<commit_message>
Checked in by casal from PC-Denis on Mon Sep  4 18:37:10 CEST 2023
</commit_message>
<xml_diff>
--- a/fsfunc.xlsx
+++ b/fsfunc.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lalannd2\MyApps\home\Sources\8-webview-test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\casal\Documents\home\5-webview-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8AB790E-F5B3-4266-A08D-633E52C279D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="73">
   <si>
     <t>absolute</t>
   </si>
@@ -248,7 +249,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -570,7 +571,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -622,6 +623,9 @@
       <c r="B5" t="s">
         <v>5</v>
       </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -646,6 +650,9 @@
       <c r="B8" t="s">
         <v>10</v>
       </c>
+      <c r="C8" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -678,6 +685,9 @@
       <c r="B12" t="s">
         <v>17</v>
       </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -711,7 +721,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -719,7 +729,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -727,15 +737,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>30</v>
       </c>
       <c r="B19" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>70</v>
       </c>
@@ -743,7 +756,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -751,7 +764,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -759,7 +772,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -767,7 +780,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -775,7 +788,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -783,7 +796,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -791,13 +804,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>72</v>
       </c>
@@ -805,7 +818,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -813,7 +826,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -821,7 +834,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>51</v>
       </c>
@@ -829,7 +842,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>53</v>
       </c>

</xml_diff>